<commit_message>
WBS through 5 October: BayanSimplify names, today's finished work, Sanad presents the pitch; spreadsheet only, as the template
</commit_message>
<xml_diff>
--- a/deliverables/02_work_breakdown_structure/Bayan_WBS.xlsx
+++ b/deliverables/02_work_breakdown_structure/Bayan_WBS.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="819" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover Page" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Cover Page" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="WBS" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1556,7 +1556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:AD76"/>
+  <dimension ref="B2:AD83"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5546875" defaultRowHeight="14.4"/>
   <cols>
     <col width="2.44140625" customWidth="1" style="1" min="1" max="1"/>
@@ -3253,7 +3253,7 @@
       <c r="B40" s="7" t="n"/>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t>3.14. Model-2 training data: 22,733 tagged, meaning-filtered pairs</t>
+          <t>3.14. BayanSimplify-v0.2 training data: 22,733 tagged, meaning-filtered pairs</t>
         </is>
       </c>
       <c r="D40" s="8" t="n"/>
@@ -3412,11 +3412,11 @@
       <c r="D43" s="8" t="n"/>
       <c r="E43" s="9" t="n"/>
       <c r="F43" s="73">
-        <f>MIN(F44:F51)</f>
+        <f>MIN(F44:F52)</f>
         <v/>
       </c>
       <c r="G43" s="73">
-        <f>MAX(G44:G51)</f>
+        <f>MAX(G44:G52)</f>
         <v/>
       </c>
       <c r="H43" s="9" t="inlineStr">
@@ -3557,7 +3557,7 @@
       <c r="B46" s="7" t="n"/>
       <c r="C46" s="8" t="inlineStr">
         <is>
-          <t>4.3. Model 1: AraT5v2 on SAMER, trained and documented (#5, #22)</t>
+          <t>4.3. BayanSimplify-v0.1: AraT5v2 on SAMER, trained and documented (#5, #22)</t>
         </is>
       </c>
       <c r="D46" s="8" t="n"/>
@@ -3575,7 +3575,7 @@
       </c>
       <c r="I46" s="10" t="inlineStr">
         <is>
-          <t>Model 1</t>
+          <t>BayanSimplify-v0.1</t>
         </is>
       </c>
       <c r="J46" s="11" t="inlineStr">
@@ -3608,7 +3608,7 @@
       <c r="B47" s="7" t="n"/>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t>4.4. Model 1 diagnosis on the locked test sets</t>
+          <t>4.4. BayanSimplify-v0.1 diagnosis on the locked test sets</t>
         </is>
       </c>
       <c r="D47" s="8" t="n"/>
@@ -3659,7 +3659,7 @@
       <c r="B48" s="7" t="n"/>
       <c r="C48" s="8" t="inlineStr">
         <is>
-          <t>4.5. Model 2 on AraT5v2 (#28, #40)</t>
+          <t>4.5. BayanSimplify-v0.2: AraT5v2 on the tagged mix (#28, #40)</t>
         </is>
       </c>
       <c r="D48" s="8" t="n"/>
@@ -3677,7 +3677,7 @@
       </c>
       <c r="I48" s="10" t="inlineStr">
         <is>
-          <t>Model 2 (AraT5v2)</t>
+          <t>BayanSimplify-v0.2</t>
         </is>
       </c>
       <c r="J48" s="11" t="inlineStr">
@@ -3710,7 +3710,7 @@
       <c r="B49" s="7" t="n"/>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>4.6. Model 2 on AraBART, and the speed benchmark (#29, #35)</t>
+          <t>4.6. BayanSimplify-v0.2-Fast: AraBART on the same mix, and the speed benchmark (#29, #35)</t>
         </is>
       </c>
       <c r="D49" s="8" t="n"/>
@@ -3728,7 +3728,7 @@
       </c>
       <c r="I49" s="10" t="inlineStr">
         <is>
-          <t>Model 2 (AraBART)</t>
+          <t>BayanSimplify-v0.2-Fast</t>
         </is>
       </c>
       <c r="J49" s="11" t="inlineStr">
@@ -3812,7 +3812,7 @@
       <c r="B51" s="7" t="n"/>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t>4.8. Model 3: AraT5v2 on corpus v1, int8 bundle (#48, #53)</t>
+          <t>4.8. BayanSimplify-v0.3: AraT5v2 on corpus v1, int8 bundle (#48, #53)</t>
         </is>
       </c>
       <c r="D51" s="8" t="n"/>
@@ -3830,7 +3830,7 @@
       </c>
       <c r="I51" s="10" t="inlineStr">
         <is>
-          <t>Model 3</t>
+          <t>BayanSimplify-v0.3</t>
         </is>
       </c>
       <c r="J51" s="11" t="inlineStr">
@@ -3860,28 +3860,30 @@
       <c r="AD51" s="14" t="n"/>
     </row>
     <row r="52" s="56">
-      <c r="B52" s="72" t="inlineStr">
-        <is>
-          <t>5. Evaluation</t>
-        </is>
-      </c>
-      <c r="C52" s="8" t="n"/>
+      <c r="B52" s="7" t="n"/>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>4.9. BayanSimplify models published on Hugging Face, with the ONNX bundles</t>
+        </is>
+      </c>
       <c r="D52" s="8" t="n"/>
       <c r="E52" s="9" t="n"/>
-      <c r="F52" s="73">
-        <f>MIN(F53:F60)</f>
-        <v/>
-      </c>
-      <c r="G52" s="73">
-        <f>MAX(G53:G60)</f>
-        <v/>
+      <c r="F52" s="73" t="n">
+        <v>46300</v>
+      </c>
+      <c r="G52" s="73" t="n">
+        <v>46300</v>
       </c>
       <c r="H52" s="9" t="inlineStr">
         <is>
-          <t>Abdul Majid, Marwan</t>
-        </is>
-      </c>
-      <c r="I52" s="10" t="inlineStr"/>
+          <t>Marwan</t>
+        </is>
+      </c>
+      <c r="I52" s="10" t="inlineStr">
+        <is>
+          <t>Public models (Hub)</t>
+        </is>
+      </c>
       <c r="J52" s="11" t="inlineStr">
         <is>
           <t>Done</t>
@@ -3909,30 +3911,28 @@
       <c r="AD52" s="14" t="n"/>
     </row>
     <row r="53" s="56">
-      <c r="B53" s="7" t="n"/>
-      <c r="C53" s="8" t="inlineStr">
-        <is>
-          <t>5.1. Scoring harness and locked test sets (#7, #15, #16, #18)</t>
-        </is>
-      </c>
+      <c r="B53" s="72" t="inlineStr">
+        <is>
+          <t>5. Evaluation</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="n"/>
       <c r="D53" s="8" t="n"/>
       <c r="E53" s="9" t="n"/>
-      <c r="F53" s="73" t="n">
-        <v>46284</v>
-      </c>
-      <c r="G53" s="73" t="n">
-        <v>46286</v>
+      <c r="F53" s="73">
+        <f>MIN(F54:F64)</f>
+        <v/>
+      </c>
+      <c r="G53" s="73">
+        <f>MAX(G54:G64)</f>
+        <v/>
       </c>
       <c r="H53" s="9" t="inlineStr">
         <is>
           <t>Abdul Majid, Marwan</t>
         </is>
       </c>
-      <c r="I53" s="10" t="inlineStr">
-        <is>
-          <t>Scripts, manifest</t>
-        </is>
-      </c>
+      <c r="I53" s="10" t="inlineStr"/>
       <c r="J53" s="11" t="inlineStr">
         <is>
           <t>Done</t>
@@ -3963,25 +3963,25 @@
       <c r="B54" s="7" t="n"/>
       <c r="C54" s="8" t="inlineStr">
         <is>
-          <t>5.2. Copy baselines, locked-set converter, generate-and-score path (#19, #24, #26)</t>
+          <t>5.1. Scoring harness and locked test sets (#7, #15, #16, #18)</t>
         </is>
       </c>
       <c r="D54" s="8" t="n"/>
       <c r="E54" s="9" t="n"/>
       <c r="F54" s="73" t="n">
+        <v>46284</v>
+      </c>
+      <c r="G54" s="73" t="n">
         <v>46286</v>
       </c>
-      <c r="G54" s="73" t="n">
-        <v>46287</v>
-      </c>
       <c r="H54" s="9" t="inlineStr">
         <is>
-          <t>Abdul Majid</t>
+          <t>Abdul Majid, Marwan</t>
         </is>
       </c>
       <c r="I54" s="10" t="inlineStr">
         <is>
-          <t>Baselines</t>
+          <t>Scripts, manifest</t>
         </is>
       </c>
       <c r="J54" s="11" t="inlineStr">
@@ -4014,25 +4014,25 @@
       <c r="B55" s="7" t="n"/>
       <c r="C55" s="8" t="inlineStr">
         <is>
-          <t>5.3. Model-2 scoring tools (#33, #34)</t>
+          <t>5.2. Copy baselines, locked-set converter, generate-and-score path (#19, #24, #26)</t>
         </is>
       </c>
       <c r="D55" s="8" t="n"/>
       <c r="E55" s="9" t="n"/>
       <c r="F55" s="73" t="n">
-        <v>46289</v>
+        <v>46286</v>
       </c>
       <c r="G55" s="73" t="n">
-        <v>46289</v>
+        <v>46287</v>
       </c>
       <c r="H55" s="9" t="inlineStr">
         <is>
-          <t>Marwan</t>
+          <t>Abdul Majid</t>
         </is>
       </c>
       <c r="I55" s="10" t="inlineStr">
         <is>
-          <t>Scoring tools</t>
+          <t>Baselines</t>
         </is>
       </c>
       <c r="J55" s="11" t="inlineStr">
@@ -4065,16 +4065,16 @@
       <c r="B56" s="7" t="n"/>
       <c r="C56" s="8" t="inlineStr">
         <is>
-          <t>5.4. BayanBench v1: behaviour tracks, document split; model 2 scored on test</t>
+          <t>5.3. BayanSimplify-v0.2 scoring tools (#33, #34)</t>
         </is>
       </c>
       <c r="D56" s="8" t="n"/>
       <c r="E56" s="9" t="n"/>
       <c r="F56" s="73" t="n">
-        <v>46291</v>
+        <v>46289</v>
       </c>
       <c r="G56" s="73" t="n">
-        <v>46293</v>
+        <v>46289</v>
       </c>
       <c r="H56" s="9" t="inlineStr">
         <is>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="I56" s="10" t="inlineStr">
         <is>
-          <t>BayanBench v1</t>
+          <t>Scoring tools</t>
         </is>
       </c>
       <c r="J56" s="11" t="inlineStr">
@@ -4116,25 +4116,25 @@
       <c r="B57" s="7" t="n"/>
       <c r="C57" s="8" t="inlineStr">
         <is>
-          <t>5.5. BayanBench v2: open meaning scorer (Gemma 4 31B); all systems scored (#48)</t>
+          <t>5.4. BayanBench v1: behaviour tracks, document split; v0.2 scored on test</t>
         </is>
       </c>
       <c r="D57" s="8" t="n"/>
       <c r="E57" s="9" t="n"/>
       <c r="F57" s="73" t="n">
-        <v>46294</v>
+        <v>46291</v>
       </c>
       <c r="G57" s="73" t="n">
-        <v>46295</v>
+        <v>46293</v>
       </c>
       <c r="H57" s="9" t="inlineStr">
         <is>
-          <t>Marwan, Abdulrahman</t>
+          <t>Marwan</t>
         </is>
       </c>
       <c r="I57" s="10" t="inlineStr">
         <is>
-          <t>BayanBench v2</t>
+          <t>BayanBench v1</t>
         </is>
       </c>
       <c r="J57" s="11" t="inlineStr">
@@ -4167,25 +4167,25 @@
       <c r="B58" s="7" t="n"/>
       <c r="C58" s="8" t="inlineStr">
         <is>
-          <t>5.6. Human rating round: 290 tasks, five raters and a reader with dyslexia (#48)</t>
+          <t>5.5. BayanBench v2: open meaning scorer (Gemma 4 31B); all systems scored (#48)</t>
         </is>
       </c>
       <c r="D58" s="8" t="n"/>
       <c r="E58" s="9" t="n"/>
       <c r="F58" s="73" t="n">
+        <v>46294</v>
+      </c>
+      <c r="G58" s="73" t="n">
         <v>46295</v>
       </c>
-      <c r="G58" s="73" t="n">
-        <v>46298</v>
-      </c>
       <c r="H58" s="9" t="inlineStr">
         <is>
-          <t>Marwan, Sanad, Ahmed, Mohammed</t>
+          <t>Marwan, Abdulrahman</t>
         </is>
       </c>
       <c r="I58" s="10" t="inlineStr">
         <is>
-          <t>Ratings, scorer check</t>
+          <t>BayanBench v2</t>
         </is>
       </c>
       <c r="J58" s="11" t="inlineStr">
@@ -4218,25 +4218,25 @@
       <c r="B59" s="7" t="n"/>
       <c r="C59" s="8" t="inlineStr">
         <is>
-          <t>5.7. BayanBench v2.0 frozen; test split scored (#55)</t>
+          <t>5.6. Human rating round: 290 tasks, five raters and a reader with dyslexia (#48)</t>
         </is>
       </c>
       <c r="D59" s="8" t="n"/>
       <c r="E59" s="9" t="n"/>
       <c r="F59" s="73" t="n">
+        <v>46295</v>
+      </c>
+      <c r="G59" s="73" t="n">
         <v>46298</v>
       </c>
-      <c r="G59" s="73" t="n">
-        <v>46299</v>
-      </c>
       <c r="H59" s="9" t="inlineStr">
         <is>
-          <t>Marwan, Abdulrahman</t>
+          <t>Marwan, Sanad, Ahmed, Mohammed</t>
         </is>
       </c>
       <c r="I59" s="10" t="inlineStr">
         <is>
-          <t>BayanBench v2.0</t>
+          <t>Ratings, scorer check</t>
         </is>
       </c>
       <c r="J59" s="11" t="inlineStr">
@@ -4269,13 +4269,13 @@
       <c r="B60" s="7" t="n"/>
       <c r="C60" s="8" t="inlineStr">
         <is>
-          <t>5.8. Model 3 ship gate and decision: an option next to model 2 (#56, #59)</t>
+          <t>5.7. BayanBench v2.0 frozen; test split scored (#55)</t>
         </is>
       </c>
       <c r="D60" s="8" t="n"/>
       <c r="E60" s="9" t="n"/>
       <c r="F60" s="73" t="n">
-        <v>46299</v>
+        <v>46298</v>
       </c>
       <c r="G60" s="73" t="n">
         <v>46299</v>
@@ -4287,7 +4287,7 @@
       </c>
       <c r="I60" s="10" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>BayanBench v2.0</t>
         </is>
       </c>
       <c r="J60" s="11" t="inlineStr">
@@ -4317,28 +4317,30 @@
       <c r="AD60" s="14" t="n"/>
     </row>
     <row r="61" s="56">
-      <c r="B61" s="72" t="inlineStr">
-        <is>
-          <t>6. Application</t>
-        </is>
-      </c>
-      <c r="C61" s="8" t="n"/>
+      <c r="B61" s="7" t="n"/>
+      <c r="C61" s="8" t="inlineStr">
+        <is>
+          <t>5.8. BayanSimplify-v0.3 ship gate; with four beams it becomes the large model (#56, #59, #68)</t>
+        </is>
+      </c>
       <c r="D61" s="8" t="n"/>
       <c r="E61" s="9" t="n"/>
-      <c r="F61" s="73">
-        <f>MIN(F62:F67)</f>
-        <v/>
-      </c>
-      <c r="G61" s="73">
-        <f>MAX(G62:G67)</f>
-        <v/>
+      <c r="F61" s="73" t="n">
+        <v>46299</v>
+      </c>
+      <c r="G61" s="73" t="n">
+        <v>46300</v>
       </c>
       <c r="H61" s="9" t="inlineStr">
         <is>
-          <t>Mohammed, Marwan</t>
-        </is>
-      </c>
-      <c r="I61" s="10" t="inlineStr"/>
+          <t>Marwan, Abdulrahman</t>
+        </is>
+      </c>
+      <c r="I61" s="10" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
       <c r="J61" s="11" t="inlineStr">
         <is>
           <t>Done</t>
@@ -4369,25 +4371,25 @@
       <c r="B62" s="7" t="n"/>
       <c r="C62" s="8" t="inlineStr">
         <is>
-          <t>6.1. PROCESS_TEXT plugin and result sheet (#14, #21)</t>
+          <t>5.9. Benchmark report: 35 systems on BayanBench v2.0 (#57, #58)</t>
         </is>
       </c>
       <c r="D62" s="8" t="n"/>
       <c r="E62" s="9" t="n"/>
       <c r="F62" s="73" t="n">
-        <v>46285</v>
+        <v>46298</v>
       </c>
       <c r="G62" s="73" t="n">
-        <v>46286</v>
+        <v>46299</v>
       </c>
       <c r="H62" s="9" t="inlineStr">
         <is>
-          <t>Mohammed</t>
+          <t>Abdulrahman</t>
         </is>
       </c>
       <c r="I62" s="10" t="inlineStr">
         <is>
-          <t>Android plugin</t>
+          <t>Benchmark report</t>
         </is>
       </c>
       <c r="J62" s="11" t="inlineStr">
@@ -4420,25 +4422,25 @@
       <c r="B63" s="7" t="n"/>
       <c r="C63" s="8" t="inlineStr">
         <is>
-          <t>6.2. Model download, result states, settings, typography (#31, #37)</t>
+          <t>5.10. Rating round for the app's three models: five raters, blind</t>
         </is>
       </c>
       <c r="D63" s="8" t="n"/>
       <c r="E63" s="9" t="n"/>
       <c r="F63" s="73" t="n">
-        <v>46289</v>
+        <v>46299</v>
       </c>
       <c r="G63" s="73" t="n">
-        <v>46295</v>
+        <v>46300</v>
       </c>
       <c r="H63" s="9" t="inlineStr">
         <is>
-          <t>Mohammed</t>
+          <t>Marwan, Sanad, Ahmed, Mohammed</t>
         </is>
       </c>
       <c r="I63" s="10" t="inlineStr">
         <is>
-          <t>App features</t>
+          <t>Ratings</t>
         </is>
       </c>
       <c r="J63" s="11" t="inlineStr">
@@ -4471,16 +4473,16 @@
       <c r="B64" s="7" t="n"/>
       <c r="C64" s="8" t="inlineStr">
         <is>
-          <t>6.3. Compose app with Material 3 Expressive (#37)</t>
+          <t>5.11. Diacritization re-benchmark: earlier numbers reproduce (#67)</t>
         </is>
       </c>
       <c r="D64" s="8" t="n"/>
       <c r="E64" s="9" t="n"/>
       <c r="F64" s="73" t="n">
-        <v>46291</v>
+        <v>46299</v>
       </c>
       <c r="G64" s="73" t="n">
-        <v>46295</v>
+        <v>46300</v>
       </c>
       <c r="H64" s="9" t="inlineStr">
         <is>
@@ -4489,7 +4491,7 @@
       </c>
       <c r="I64" s="10" t="inlineStr">
         <is>
-          <t>App</t>
+          <t>Re-benchmark</t>
         </is>
       </c>
       <c r="J64" s="11" t="inlineStr">
@@ -4519,30 +4521,28 @@
       <c r="AD64" s="14" t="n"/>
     </row>
     <row r="65" s="56">
-      <c r="B65" s="7" t="n"/>
-      <c r="C65" s="8" t="inlineStr">
-        <is>
-          <t>6.4. Read-aloud with word highlighting (Nabra through sherpa-onnx)</t>
-        </is>
-      </c>
+      <c r="B65" s="72" t="inlineStr">
+        <is>
+          <t>6. Application</t>
+        </is>
+      </c>
+      <c r="C65" s="8" t="n"/>
       <c r="D65" s="8" t="n"/>
       <c r="E65" s="9" t="n"/>
-      <c r="F65" s="73" t="n">
-        <v>46292</v>
-      </c>
-      <c r="G65" s="73" t="n">
-        <v>46295</v>
+      <c r="F65" s="73">
+        <f>MIN(F66:F74)</f>
+        <v/>
+      </c>
+      <c r="G65" s="73">
+        <f>MAX(G66:G74)</f>
+        <v/>
       </c>
       <c r="H65" s="9" t="inlineStr">
         <is>
-          <t>Marwan</t>
-        </is>
-      </c>
-      <c r="I65" s="10" t="inlineStr">
-        <is>
-          <t>Read-aloud</t>
-        </is>
-      </c>
+          <t>Mohammed, Marwan</t>
+        </is>
+      </c>
+      <c r="I65" s="10" t="inlineStr"/>
       <c r="J65" s="11" t="inlineStr">
         <is>
           <t>Done</t>
@@ -4573,25 +4573,25 @@
       <c r="B66" s="7" t="n"/>
       <c r="C66" s="8" t="inlineStr">
         <is>
-          <t>6.5. Overlay, floating reader, text-step guards, Bayan design system (#54)</t>
+          <t>6.1. PROCESS_TEXT plugin and result sheet (#14, #21)</t>
         </is>
       </c>
       <c r="D66" s="8" t="n"/>
       <c r="E66" s="9" t="n"/>
       <c r="F66" s="73" t="n">
-        <v>46296</v>
+        <v>46285</v>
       </c>
       <c r="G66" s="73" t="n">
-        <v>46299</v>
+        <v>46286</v>
       </c>
       <c r="H66" s="9" t="inlineStr">
         <is>
-          <t>Marwan</t>
+          <t>Mohammed</t>
         </is>
       </c>
       <c r="I66" s="10" t="inlineStr">
         <is>
-          <t>App release</t>
+          <t>Android plugin</t>
         </is>
       </c>
       <c r="J66" s="11" t="inlineStr">
@@ -4624,25 +4624,25 @@
       <c r="B67" s="7" t="n"/>
       <c r="C67" s="8" t="inlineStr">
         <is>
-          <t>6.6. Beam search as a per-model decoding option (#61, #62)</t>
+          <t>6.2. Model download, result states, settings, typography (#31, #37)</t>
         </is>
       </c>
       <c r="D67" s="8" t="n"/>
       <c r="E67" s="9" t="n"/>
       <c r="F67" s="73" t="n">
-        <v>46299</v>
+        <v>46289</v>
       </c>
       <c r="G67" s="73" t="n">
-        <v>46299</v>
+        <v>46295</v>
       </c>
       <c r="H67" s="9" t="inlineStr">
         <is>
-          <t>Marwan</t>
+          <t>Mohammed</t>
         </is>
       </c>
       <c r="I67" s="10" t="inlineStr">
         <is>
-          <t>Decoder</t>
+          <t>App features</t>
         </is>
       </c>
       <c r="J67" s="11" t="inlineStr">
@@ -4672,28 +4672,30 @@
       <c r="AD67" s="14" t="n"/>
     </row>
     <row r="68" s="56">
-      <c r="B68" s="72" t="inlineStr">
-        <is>
-          <t>7. On-device model</t>
-        </is>
-      </c>
-      <c r="C68" s="8" t="n"/>
+      <c r="B68" s="7" t="n"/>
+      <c r="C68" s="8" t="inlineStr">
+        <is>
+          <t>6.3. Compose app with Material 3 Expressive (#37)</t>
+        </is>
+      </c>
       <c r="D68" s="8" t="n"/>
       <c r="E68" s="9" t="n"/>
-      <c r="F68" s="73">
-        <f>MIN(F69:F70)</f>
-        <v/>
-      </c>
-      <c r="G68" s="73">
-        <f>MAX(G69:G70)</f>
-        <v/>
+      <c r="F68" s="73" t="n">
+        <v>46291</v>
+      </c>
+      <c r="G68" s="73" t="n">
+        <v>46295</v>
       </c>
       <c r="H68" s="9" t="inlineStr">
         <is>
           <t>Marwan</t>
         </is>
       </c>
-      <c r="I68" s="10" t="inlineStr"/>
+      <c r="I68" s="10" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
       <c r="J68" s="11" t="inlineStr">
         <is>
           <t>Done</t>
@@ -4724,16 +4726,16 @@
       <c r="B69" s="7" t="n"/>
       <c r="C69" s="8" t="inlineStr">
         <is>
-          <t>7.1. ONNX export, int8 quantization, on-device engine (#32)</t>
+          <t>6.4. Read-aloud with word highlighting (Nabra through sherpa-onnx)</t>
         </is>
       </c>
       <c r="D69" s="8" t="n"/>
       <c r="E69" s="9" t="n"/>
       <c r="F69" s="73" t="n">
-        <v>46289</v>
+        <v>46292</v>
       </c>
       <c r="G69" s="73" t="n">
-        <v>46291</v>
+        <v>46295</v>
       </c>
       <c r="H69" s="9" t="inlineStr">
         <is>
@@ -4742,7 +4744,7 @@
       </c>
       <c r="I69" s="10" t="inlineStr">
         <is>
-          <t>Model bundles</t>
+          <t>Read-aloud</t>
         </is>
       </c>
       <c r="J69" s="11" t="inlineStr">
@@ -4775,13 +4777,13 @@
       <c r="B70" s="7" t="n"/>
       <c r="C70" s="8" t="inlineStr">
         <is>
-          <t>7.2. Phone latency: AraT5v2 (26 Sep), AraBART (3 Oct), beam search (4 Oct)</t>
+          <t>6.5. Overlay, floating reader, text-step guards, Bayan design system (#54)</t>
         </is>
       </c>
       <c r="D70" s="8" t="n"/>
       <c r="E70" s="9" t="n"/>
       <c r="F70" s="73" t="n">
-        <v>46291</v>
+        <v>46296</v>
       </c>
       <c r="G70" s="73" t="n">
         <v>46299</v>
@@ -4793,7 +4795,7 @@
       </c>
       <c r="I70" s="10" t="inlineStr">
         <is>
-          <t>Measurements</t>
+          <t>App release</t>
         </is>
       </c>
       <c r="J70" s="11" t="inlineStr">
@@ -4823,31 +4825,33 @@
       <c r="AD70" s="14" t="n"/>
     </row>
     <row r="71" s="56">
-      <c r="B71" s="72" t="inlineStr">
-        <is>
-          <t>8. Final deliverables</t>
-        </is>
-      </c>
-      <c r="C71" s="8" t="n"/>
+      <c r="B71" s="7" t="n"/>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>6.6. Beam search as a per-model decoding option (#61, #62)</t>
+        </is>
+      </c>
       <c r="D71" s="8" t="n"/>
       <c r="E71" s="9" t="n"/>
-      <c r="F71" s="73">
-        <f>MIN(F72:F76)</f>
-        <v/>
-      </c>
-      <c r="G71" s="73">
-        <f>MAX(G72:G76)</f>
-        <v/>
+      <c r="F71" s="73" t="n">
+        <v>46299</v>
+      </c>
+      <c r="G71" s="73" t="n">
+        <v>46299</v>
       </c>
       <c r="H71" s="9" t="inlineStr">
         <is>
-          <t>Marwan, Abdulrahman</t>
-        </is>
-      </c>
-      <c r="I71" s="10" t="inlineStr"/>
+          <t>Marwan</t>
+        </is>
+      </c>
+      <c r="I71" s="10" t="inlineStr">
+        <is>
+          <t>Decoder</t>
+        </is>
+      </c>
       <c r="J71" s="11" t="inlineStr">
         <is>
-          <t>In-progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K71" s="7" t="n"/>
@@ -4875,30 +4879,30 @@
       <c r="B72" s="7" t="n"/>
       <c r="C72" s="8" t="inlineStr">
         <is>
-          <t>8.1. Final report (#52)</t>
+          <t>6.7. BayanSimplify-v0.3 as the large model, four beams on by default; safety net (#66)</t>
         </is>
       </c>
       <c r="D72" s="8" t="n"/>
       <c r="E72" s="9" t="n"/>
       <c r="F72" s="73" t="n">
-        <v>46294</v>
+        <v>46299</v>
       </c>
       <c r="G72" s="73" t="n">
         <v>46300</v>
       </c>
       <c r="H72" s="9" t="inlineStr">
         <is>
-          <t>Marwan, Abdulrahman</t>
+          <t>Marwan</t>
         </is>
       </c>
       <c r="I72" s="10" t="inlineStr">
         <is>
-          <t>Final report</t>
+          <t>App release</t>
         </is>
       </c>
       <c r="J72" s="11" t="inlineStr">
         <is>
-          <t>In-progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K72" s="7" t="n"/>
@@ -4926,30 +4930,30 @@
       <c r="B73" s="7" t="n"/>
       <c r="C73" s="8" t="inlineStr">
         <is>
-          <t>8.2. Presentation deck (#50)</t>
+          <t>6.8. Tashkeel in the app: Libtashkeel bundled (#67)</t>
         </is>
       </c>
       <c r="D73" s="8" t="n"/>
       <c r="E73" s="9" t="n"/>
       <c r="F73" s="73" t="n">
-        <v>46297</v>
+        <v>46299</v>
       </c>
       <c r="G73" s="73" t="n">
         <v>46300</v>
       </c>
       <c r="H73" s="9" t="inlineStr">
         <is>
-          <t>Abdulrahman</t>
+          <t>Marwan</t>
         </is>
       </c>
       <c r="I73" s="10" t="inlineStr">
         <is>
-          <t>Slide deck</t>
+          <t>Tashkeel setting</t>
         </is>
       </c>
       <c r="J73" s="11" t="inlineStr">
         <is>
-          <t>In-progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K73" s="7" t="n"/>
@@ -4977,13 +4981,13 @@
       <c r="B74" s="7" t="n"/>
       <c r="C74" s="8" t="inlineStr">
         <is>
-          <t>8.3. Coding reference: repository and README (#60)</t>
+          <t>6.9. Design system in the repository (#69)</t>
         </is>
       </c>
       <c r="D74" s="8" t="n"/>
       <c r="E74" s="9" t="n"/>
       <c r="F74" s="73" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="G74" s="73" t="n">
         <v>46300</v>
@@ -4995,12 +4999,12 @@
       </c>
       <c r="I74" s="10" t="inlineStr">
         <is>
-          <t>Repository</t>
+          <t>Design system</t>
         </is>
       </c>
       <c r="J74" s="11" t="inlineStr">
         <is>
-          <t>In-progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K74" s="7" t="n"/>
@@ -5025,27 +5029,33 @@
       <c r="AD74" s="14" t="n"/>
     </row>
     <row r="75" s="56">
-      <c r="B75" s="7" t="n"/>
-      <c r="C75" s="8" t="inlineStr">
-        <is>
-          <t>8.4. Demo video</t>
-        </is>
-      </c>
+      <c r="B75" s="72" t="inlineStr">
+        <is>
+          <t>7. On-device model</t>
+        </is>
+      </c>
+      <c r="C75" s="8" t="n"/>
       <c r="D75" s="8" t="n"/>
       <c r="E75" s="9" t="n"/>
-      <c r="F75" s="73" t="n"/>
-      <c r="G75" s="73" t="n"/>
+      <c r="F75" s="73">
+        <f>MIN(F76:F77)</f>
+        <v/>
+      </c>
+      <c r="G75" s="73">
+        <f>MAX(G76:G77)</f>
+        <v/>
+      </c>
       <c r="H75" s="9" t="inlineStr">
         <is>
           <t>Marwan</t>
         </is>
       </c>
-      <c r="I75" s="10" t="inlineStr">
-        <is>
-          <t>Demo video</t>
-        </is>
-      </c>
-      <c r="J75" s="11" t="n"/>
+      <c r="I75" s="10" t="inlineStr"/>
+      <c r="J75" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="K75" s="7" t="n"/>
       <c r="L75" s="8" t="n"/>
       <c r="M75" s="8" t="n"/>
@@ -5071,24 +5081,32 @@
       <c r="B76" s="7" t="n"/>
       <c r="C76" s="8" t="inlineStr">
         <is>
-          <t>8.5. Final pitch (Tue 6 Oct)</t>
+          <t>7.1. ONNX export, int8 quantization, on-device engine (#32)</t>
         </is>
       </c>
       <c r="D76" s="8" t="n"/>
       <c r="E76" s="9" t="n"/>
-      <c r="F76" s="73" t="n"/>
-      <c r="G76" s="73" t="n"/>
+      <c r="F76" s="73" t="n">
+        <v>46289</v>
+      </c>
+      <c r="G76" s="73" t="n">
+        <v>46291</v>
+      </c>
       <c r="H76" s="9" t="inlineStr">
         <is>
-          <t>Marwan, Abdulrahman</t>
+          <t>Marwan</t>
         </is>
       </c>
       <c r="I76" s="10" t="inlineStr">
         <is>
-          <t>Pitch</t>
-        </is>
-      </c>
-      <c r="J76" s="11" t="n"/>
+          <t>Model bundles</t>
+        </is>
+      </c>
+      <c r="J76" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="K76" s="7" t="n"/>
       <c r="L76" s="8" t="n"/>
       <c r="M76" s="8" t="n"/>
@@ -5110,6 +5128,345 @@
       <c r="AC76" s="8" t="n"/>
       <c r="AD76" s="14" t="n"/>
     </row>
+    <row r="77" s="56">
+      <c r="B77" s="7" t="n"/>
+      <c r="C77" s="8" t="inlineStr">
+        <is>
+          <t>7.2. Phone latency: AraT5v2 (26 Sep), AraBART (3 Oct), beam search (4 Oct)</t>
+        </is>
+      </c>
+      <c r="D77" s="8" t="n"/>
+      <c r="E77" s="9" t="n"/>
+      <c r="F77" s="73" t="n">
+        <v>46291</v>
+      </c>
+      <c r="G77" s="73" t="n">
+        <v>46299</v>
+      </c>
+      <c r="H77" s="9" t="inlineStr">
+        <is>
+          <t>Marwan</t>
+        </is>
+      </c>
+      <c r="I77" s="10" t="inlineStr">
+        <is>
+          <t>Measurements</t>
+        </is>
+      </c>
+      <c r="J77" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K77" s="7" t="n"/>
+      <c r="L77" s="8" t="n"/>
+      <c r="M77" s="8" t="n"/>
+      <c r="N77" s="8" t="n"/>
+      <c r="O77" s="8" t="n"/>
+      <c r="P77" s="8" t="n"/>
+      <c r="Q77" s="8" t="n"/>
+      <c r="R77" s="8" t="n"/>
+      <c r="S77" s="8" t="n"/>
+      <c r="T77" s="8" t="n"/>
+      <c r="U77" s="8" t="n"/>
+      <c r="V77" s="8" t="n"/>
+      <c r="W77" s="8" t="n"/>
+      <c r="X77" s="8" t="n"/>
+      <c r="Y77" s="8" t="n"/>
+      <c r="Z77" s="8" t="n"/>
+      <c r="AA77" s="8" t="n"/>
+      <c r="AB77" s="8" t="n"/>
+      <c r="AC77" s="8" t="n"/>
+      <c r="AD77" s="14" t="n"/>
+    </row>
+    <row r="78" s="56">
+      <c r="B78" s="72" t="inlineStr">
+        <is>
+          <t>8. Final deliverables</t>
+        </is>
+      </c>
+      <c r="C78" s="8" t="n"/>
+      <c r="D78" s="8" t="n"/>
+      <c r="E78" s="9" t="n"/>
+      <c r="F78" s="73">
+        <f>MIN(F79:F83)</f>
+        <v/>
+      </c>
+      <c r="G78" s="73">
+        <f>MAX(G79:G83)</f>
+        <v/>
+      </c>
+      <c r="H78" s="9" t="inlineStr">
+        <is>
+          <t>Marwan, Abdulrahman</t>
+        </is>
+      </c>
+      <c r="I78" s="10" t="inlineStr"/>
+      <c r="J78" s="11" t="inlineStr">
+        <is>
+          <t>In-progress</t>
+        </is>
+      </c>
+      <c r="K78" s="7" t="n"/>
+      <c r="L78" s="8" t="n"/>
+      <c r="M78" s="8" t="n"/>
+      <c r="N78" s="8" t="n"/>
+      <c r="O78" s="8" t="n"/>
+      <c r="P78" s="8" t="n"/>
+      <c r="Q78" s="8" t="n"/>
+      <c r="R78" s="8" t="n"/>
+      <c r="S78" s="8" t="n"/>
+      <c r="T78" s="8" t="n"/>
+      <c r="U78" s="8" t="n"/>
+      <c r="V78" s="8" t="n"/>
+      <c r="W78" s="8" t="n"/>
+      <c r="X78" s="8" t="n"/>
+      <c r="Y78" s="8" t="n"/>
+      <c r="Z78" s="8" t="n"/>
+      <c r="AA78" s="8" t="n"/>
+      <c r="AB78" s="8" t="n"/>
+      <c r="AC78" s="8" t="n"/>
+      <c r="AD78" s="14" t="n"/>
+    </row>
+    <row r="79" s="56">
+      <c r="B79" s="7" t="n"/>
+      <c r="C79" s="8" t="inlineStr">
+        <is>
+          <t>8.1. Final report (#52, #70)</t>
+        </is>
+      </c>
+      <c r="D79" s="8" t="n"/>
+      <c r="E79" s="9" t="n"/>
+      <c r="F79" s="73" t="n">
+        <v>46294</v>
+      </c>
+      <c r="G79" s="73" t="n">
+        <v>46300</v>
+      </c>
+      <c r="H79" s="9" t="inlineStr">
+        <is>
+          <t>Marwan, Abdulrahman</t>
+        </is>
+      </c>
+      <c r="I79" s="10" t="inlineStr">
+        <is>
+          <t>Final report</t>
+        </is>
+      </c>
+      <c r="J79" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K79" s="7" t="n"/>
+      <c r="L79" s="8" t="n"/>
+      <c r="M79" s="8" t="n"/>
+      <c r="N79" s="8" t="n"/>
+      <c r="O79" s="8" t="n"/>
+      <c r="P79" s="8" t="n"/>
+      <c r="Q79" s="8" t="n"/>
+      <c r="R79" s="8" t="n"/>
+      <c r="S79" s="8" t="n"/>
+      <c r="T79" s="8" t="n"/>
+      <c r="U79" s="8" t="n"/>
+      <c r="V79" s="8" t="n"/>
+      <c r="W79" s="8" t="n"/>
+      <c r="X79" s="8" t="n"/>
+      <c r="Y79" s="8" t="n"/>
+      <c r="Z79" s="8" t="n"/>
+      <c r="AA79" s="8" t="n"/>
+      <c r="AB79" s="8" t="n"/>
+      <c r="AC79" s="8" t="n"/>
+      <c r="AD79" s="14" t="n"/>
+    </row>
+    <row r="80" s="56">
+      <c r="B80" s="7" t="n"/>
+      <c r="C80" s="8" t="inlineStr">
+        <is>
+          <t>8.2. Pitch deck (#50)</t>
+        </is>
+      </c>
+      <c r="D80" s="8" t="n"/>
+      <c r="E80" s="9" t="n"/>
+      <c r="F80" s="73" t="n">
+        <v>46297</v>
+      </c>
+      <c r="G80" s="73" t="n">
+        <v>46300</v>
+      </c>
+      <c r="H80" s="9" t="inlineStr">
+        <is>
+          <t>Abdulrahman</t>
+        </is>
+      </c>
+      <c r="I80" s="10" t="inlineStr">
+        <is>
+          <t>Slide deck</t>
+        </is>
+      </c>
+      <c r="J80" s="11" t="inlineStr">
+        <is>
+          <t>In-progress</t>
+        </is>
+      </c>
+      <c r="K80" s="7" t="n"/>
+      <c r="L80" s="8" t="n"/>
+      <c r="M80" s="8" t="n"/>
+      <c r="N80" s="8" t="n"/>
+      <c r="O80" s="8" t="n"/>
+      <c r="P80" s="8" t="n"/>
+      <c r="Q80" s="8" t="n"/>
+      <c r="R80" s="8" t="n"/>
+      <c r="S80" s="8" t="n"/>
+      <c r="T80" s="8" t="n"/>
+      <c r="U80" s="8" t="n"/>
+      <c r="V80" s="8" t="n"/>
+      <c r="W80" s="8" t="n"/>
+      <c r="X80" s="8" t="n"/>
+      <c r="Y80" s="8" t="n"/>
+      <c r="Z80" s="8" t="n"/>
+      <c r="AA80" s="8" t="n"/>
+      <c r="AB80" s="8" t="n"/>
+      <c r="AC80" s="8" t="n"/>
+      <c r="AD80" s="14" t="n"/>
+    </row>
+    <row r="81" s="56">
+      <c r="B81" s="7" t="n"/>
+      <c r="C81" s="8" t="inlineStr">
+        <is>
+          <t>8.3. Coding reference: repository and README (#60, #70)</t>
+        </is>
+      </c>
+      <c r="D81" s="8" t="n"/>
+      <c r="E81" s="9" t="n"/>
+      <c r="F81" s="73" t="n">
+        <v>46299</v>
+      </c>
+      <c r="G81" s="73" t="n">
+        <v>46300</v>
+      </c>
+      <c r="H81" s="9" t="inlineStr">
+        <is>
+          <t>Marwan</t>
+        </is>
+      </c>
+      <c r="I81" s="10" t="inlineStr">
+        <is>
+          <t>Repository</t>
+        </is>
+      </c>
+      <c r="J81" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K81" s="7" t="n"/>
+      <c r="L81" s="8" t="n"/>
+      <c r="M81" s="8" t="n"/>
+      <c r="N81" s="8" t="n"/>
+      <c r="O81" s="8" t="n"/>
+      <c r="P81" s="8" t="n"/>
+      <c r="Q81" s="8" t="n"/>
+      <c r="R81" s="8" t="n"/>
+      <c r="S81" s="8" t="n"/>
+      <c r="T81" s="8" t="n"/>
+      <c r="U81" s="8" t="n"/>
+      <c r="V81" s="8" t="n"/>
+      <c r="W81" s="8" t="n"/>
+      <c r="X81" s="8" t="n"/>
+      <c r="Y81" s="8" t="n"/>
+      <c r="Z81" s="8" t="n"/>
+      <c r="AA81" s="8" t="n"/>
+      <c r="AB81" s="8" t="n"/>
+      <c r="AC81" s="8" t="n"/>
+      <c r="AD81" s="14" t="n"/>
+    </row>
+    <row r="82" s="56">
+      <c r="B82" s="7" t="n"/>
+      <c r="C82" s="8" t="inlineStr">
+        <is>
+          <t>8.4. Demo video</t>
+        </is>
+      </c>
+      <c r="D82" s="8" t="n"/>
+      <c r="E82" s="9" t="n"/>
+      <c r="F82" s="73" t="n"/>
+      <c r="G82" s="73" t="n"/>
+      <c r="H82" s="9" t="inlineStr">
+        <is>
+          <t>Marwan</t>
+        </is>
+      </c>
+      <c r="I82" s="10" t="inlineStr">
+        <is>
+          <t>Demo video</t>
+        </is>
+      </c>
+      <c r="J82" s="11" t="n"/>
+      <c r="K82" s="7" t="n"/>
+      <c r="L82" s="8" t="n"/>
+      <c r="M82" s="8" t="n"/>
+      <c r="N82" s="8" t="n"/>
+      <c r="O82" s="8" t="n"/>
+      <c r="P82" s="8" t="n"/>
+      <c r="Q82" s="8" t="n"/>
+      <c r="R82" s="8" t="n"/>
+      <c r="S82" s="8" t="n"/>
+      <c r="T82" s="8" t="n"/>
+      <c r="U82" s="8" t="n"/>
+      <c r="V82" s="8" t="n"/>
+      <c r="W82" s="8" t="n"/>
+      <c r="X82" s="8" t="n"/>
+      <c r="Y82" s="8" t="n"/>
+      <c r="Z82" s="8" t="n"/>
+      <c r="AA82" s="8" t="n"/>
+      <c r="AB82" s="8" t="n"/>
+      <c r="AC82" s="8" t="n"/>
+      <c r="AD82" s="14" t="n"/>
+    </row>
+    <row r="83" s="56">
+      <c r="B83" s="7" t="n"/>
+      <c r="C83" s="8" t="inlineStr">
+        <is>
+          <t>8.5. Final pitch (Tue 6 Oct), presented by Sanad</t>
+        </is>
+      </c>
+      <c r="D83" s="8" t="n"/>
+      <c r="E83" s="9" t="n"/>
+      <c r="F83" s="73" t="n"/>
+      <c r="G83" s="73" t="n"/>
+      <c r="H83" s="9" t="inlineStr">
+        <is>
+          <t>Sanad</t>
+        </is>
+      </c>
+      <c r="I83" s="10" t="inlineStr">
+        <is>
+          <t>Pitch</t>
+        </is>
+      </c>
+      <c r="J83" s="11" t="n"/>
+      <c r="K83" s="7" t="n"/>
+      <c r="L83" s="8" t="n"/>
+      <c r="M83" s="8" t="n"/>
+      <c r="N83" s="8" t="n"/>
+      <c r="O83" s="8" t="n"/>
+      <c r="P83" s="8" t="n"/>
+      <c r="Q83" s="8" t="n"/>
+      <c r="R83" s="8" t="n"/>
+      <c r="S83" s="8" t="n"/>
+      <c r="T83" s="8" t="n"/>
+      <c r="U83" s="8" t="n"/>
+      <c r="V83" s="8" t="n"/>
+      <c r="W83" s="8" t="n"/>
+      <c r="X83" s="8" t="n"/>
+      <c r="Y83" s="8" t="n"/>
+      <c r="Z83" s="8" t="n"/>
+      <c r="AA83" s="8" t="n"/>
+      <c r="AB83" s="8" t="n"/>
+      <c r="AC83" s="8" t="n"/>
+      <c r="AD83" s="14" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="K11:O11"/>
@@ -5314,12 +5671,12 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K52:AD52">
-    <cfRule type="expression" priority="39" dxfId="0">
+    <cfRule type="expression" priority="39" dxfId="1">
       <formula>AND(K$13&gt;=$F52,K$13&lt;=$G52)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K53:AD53">
-    <cfRule type="expression" priority="40" dxfId="1">
+    <cfRule type="expression" priority="40" dxfId="0">
       <formula>AND(K$13&gt;=$F53,K$13&lt;=$G53)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5359,7 +5716,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K61:AD61">
-    <cfRule type="expression" priority="48" dxfId="0">
+    <cfRule type="expression" priority="48" dxfId="1">
       <formula>AND(K$13&gt;=$F61,K$13&lt;=$G61)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5379,7 +5736,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K65:AD65">
-    <cfRule type="expression" priority="52" dxfId="1">
+    <cfRule type="expression" priority="52" dxfId="0">
       <formula>AND(K$13&gt;=$F65,K$13&lt;=$G65)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5394,7 +5751,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K68:AD68">
-    <cfRule type="expression" priority="55" dxfId="0">
+    <cfRule type="expression" priority="55" dxfId="1">
       <formula>AND(K$13&gt;=$F68,K$13&lt;=$G68)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5409,7 +5766,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K71:AD71">
-    <cfRule type="expression" priority="58" dxfId="0">
+    <cfRule type="expression" priority="58" dxfId="1">
       <formula>AND(K$13&gt;=$F71,K$13&lt;=$G71)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5429,7 +5786,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K75:AD75">
-    <cfRule type="expression" priority="62" dxfId="1">
+    <cfRule type="expression" priority="62" dxfId="0">
       <formula>AND(K$13&gt;=$F75,K$13&lt;=$G75)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5438,8 +5795,43 @@
       <formula>AND(K$13&gt;=$F76,K$13&lt;=$G76)</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="K77:AD77">
+    <cfRule type="expression" priority="64" dxfId="1">
+      <formula>AND(K$13&gt;=$F77,K$13&lt;=$G77)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K78:AD78">
+    <cfRule type="expression" priority="65" dxfId="0">
+      <formula>AND(K$13&gt;=$F78,K$13&lt;=$G78)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K79:AD79">
+    <cfRule type="expression" priority="66" dxfId="1">
+      <formula>AND(K$13&gt;=$F79,K$13&lt;=$G79)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K80:AD80">
+    <cfRule type="expression" priority="67" dxfId="1">
+      <formula>AND(K$13&gt;=$F80,K$13&lt;=$G80)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K81:AD81">
+    <cfRule type="expression" priority="68" dxfId="1">
+      <formula>AND(K$13&gt;=$F81,K$13&lt;=$G81)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K82:AD82">
+    <cfRule type="expression" priority="69" dxfId="1">
+      <formula>AND(K$13&gt;=$F82,K$13&lt;=$G82)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K83:AD83">
+    <cfRule type="expression" priority="70" dxfId="1">
+      <formula>AND(K$13&gt;=$F83,K$13&lt;=$G83)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="J14:J76" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="J14:J83" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>$J$3:$J$5</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>